<commit_message>
Update sport to be able to configure the name of the roster column on sport draws (Umpire or Scorer)
</commit_message>
<xml_diff>
--- a/test/fixtures/files/invalid_sport.xlsx
+++ b/test/fixtures/files/invalid_sport.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>Name</t>
   </si>
@@ -52,6 +52,9 @@
     <t>AllowNeg</t>
   </si>
   <si>
+    <t>UmpireText</t>
+  </si>
+  <si>
     <t>PointName</t>
   </si>
   <si>
@@ -71,6 +74,9 @@
   </si>
   <si>
     <t>false</t>
+  </si>
+  <si>
+    <t>Umpire</t>
   </si>
   <si>
     <t>Point</t>
@@ -91,7 +97,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -123,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -131,14 +137,20 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -442,25 +454,26 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="6.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="6.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="10.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="4" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="4" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="4" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="4" width="10.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="6.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="6.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="10.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="10.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -497,49 +510,55 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>99</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="3">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3">
-        <v>99</v>
-      </c>
-      <c r="F2" s="3">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="3">
+        <v>15</v>
+      </c>
+      <c r="J2" s="4">
         <v>5</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2" s="1" t="s">
         <v>19</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>